<commit_message>
Executed on July 25
</commit_message>
<xml_diff>
--- a/Encollect_Web_SCB_P3/Cypress/fixtures/UnAllocation_acclevel.xlsx
+++ b/Encollect_Web_SCB_P3/Cypress/fixtures/UnAllocation_acclevel.xlsx
@@ -32,11 +32,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:vt="http://schemas.openxmlformats.org/officeDocument/2006/docPropsVTypes">
-  <numFmts count="4">
+  <numFmts count="2">
     <numFmt numFmtId="56" formatCode="&quot;上午/下午 &quot;hh&quot;時&quot;mm&quot;分&quot;ss&quot;秒 &quot;"/>
-    <numFmt numFmtId="164" formatCode="General"/>
-    <numFmt numFmtId="165" formatCode="@"/>
-    <numFmt numFmtId="166" formatCode="d\ mmm\ yy"/>
+    <numFmt numFmtId="164" formatCode="d\ mmm\ yy"/>
   </numFmts>
   <fonts count="1">
     <font>
@@ -67,9 +65,8 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -404,7 +401,7 @@
   <dimension ref="A1:A2"/>
   <sheetData>
     <row r="2">
-      <c r="A2" s="1" t="str">
+      <c r="A2" t="str">
         <v>10008932</v>
       </c>
     </row>

</xml_diff>